<commit_message>
Update Martabe reference matrix with SWI 204
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0121qocWgsZdFAsne2oz9sHT
</commit_message>
<xml_diff>
--- a/Matriks-Rujukan-Martabe-SWI-201-203.xlsx
+++ b/Matriks-Rujukan-Martabe-SWI-201-203.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -729,7 +729,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>201-003, 203-002</t>
+          <t>201-003, 203-002, 204-004</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>201-021</t>
+          <t>201-021, 204-001</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>201-021</t>
+          <t>201-021, 204-001</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>203-003</t>
+          <t>203-003, 204-002</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>203-003</t>
+          <t>203-003, 204-002</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>203-010</t>
+          <t>203-010, 204-002</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>203-002</t>
+          <t>203-002, 204-004</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1698,6 +1698,66 @@
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Menunggu dokumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>KBK-MIR-LAB-PRE-SOP-008</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Uji Kehalusan Sampel</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>204-002</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Menunggu dokumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>KBK-MIR-MP-PRO-OPE-SOP-0015</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>SG solid determination by pycnometer</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>204-005</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Menunggu dokumen</t>
         </is>
@@ -1714,7 +1774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1898,6 +1958,18 @@
       <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Tidak ada rujukan SOP Martabe; perlu dicek apakah Martabe punya padanannya</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>204-003</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>'No source held'; laser sizer tidak ada di quotation ILS Q0023979 - perlu dicek apakah alatnya ada</t>
         </is>
       </c>
     </row>
@@ -1963,7 +2035,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Total: 43 dokumen Martabe (41 baris; 0039/0040 dan 0041/0042 digabung per baris); 37 SWI diperiksa (201-001..025, 203-001..012).</t>
+          <t>Total: 45 dokumen Martabe (43 baris; 0039/0040 dan 0041/0042 digabung per baris); 42 SWI diperiksa (201-001..025, 203-001..012, 204-001..005).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Martabe reference matrix with SWI 204-006..010
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0121qocWgsZdFAsne2oz9sHT
</commit_message>
<xml_diff>
--- a/Matriks-Rujukan-Martabe-SWI-201-203.xlsx
+++ b/Matriks-Rujukan-Martabe-SWI-201-203.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>203-007</t>
+          <t>203-007, 204-009</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1758,6 +1758,156 @@
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Menunggu dokumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>KBK-MIR-MP-PRO-OPE-SOP-0022</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Moisture Content</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>204-006</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Menunggu dokumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>KBK-MIR-MP-PRO-MET-SOP-0032</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Moisture Content (master Bahasa)</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>204-006</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Menunggu dokumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>KBK-MIR-MP-PRO-OPE-SOP-0017</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Total Suspended Solid</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>204-007</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Menunggu dokumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>KBK-MIR-LAB-ENV-SOP-072</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Analisa TSS Gravimetri</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>204-007</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Menunggu dokumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>KBK-MIR-MP-PRO-OPE-SOP-0016</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Uji Viskositas</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>204-008</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>Menunggu dokumen</t>
         </is>
@@ -1774,7 +1924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1970,6 +2120,18 @@
       <c r="B16" t="inlineStr">
         <is>
           <t>'No source held'; laser sizer tidak ada di quotation ILS Q0023979 - perlu dicek apakah alatnya ada</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>204-010</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Hanya rujukan vendor (control philosophy Roytec); tidak ada rujukan SOP Martabe</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2197,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Total: 45 dokumen Martabe (43 baris; 0039/0040 dan 0041/0042 digabung per baris); 42 SWI diperiksa (201-001..025, 203-001..012, 204-001..005).</t>
+          <t>Total: 50 dokumen Martabe (48 baris; 0039/0040 dan 0041/0042 digabung per baris); 47 SWI diperiksa (201-001..025, 203-001..012, 204-001..010).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Martabe reference matrix with SWI 204-011..015
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0121qocWgsZdFAsne2oz9sHT
</commit_message>
<xml_diff>
--- a/Matriks-Rujukan-Martabe-SWI-201-203.xlsx
+++ b/Matriks-Rujukan-Martabe-SWI-201-203.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -789,7 +789,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>201-011, 201-012, 203-006, 203-011</t>
+          <t>201-011, 201-012, 203-006, 203-011, 204-015</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>201-005</t>
+          <t>201-005, 204-014</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>203-001</t>
+          <t>203-001, 204-013</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>201-014, 201-015</t>
+          <t>201-014, 201-015, 204-011</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -1908,6 +1908,96 @@
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Menunggu dokumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>KBK-MIR-MP-PRO-OPE-SOP-0023</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Filter Press</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>204-011</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Menunggu dokumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>KBK-MIR-MP-PRO-OPE-SOP-0006</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Uji Bond Work Index (BWI)</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>204-012</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Menunggu dokumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>KBK-MIR-MP-PRO-OPE-SOP-0012</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Uji Pengujian Grind Establishment</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>204-013</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Menunggu dokumen</t>
         </is>
@@ -2197,7 +2287,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Total: 50 dokumen Martabe (48 baris; 0039/0040 dan 0041/0042 digabung per baris); 47 SWI diperiksa (201-001..025, 203-001..012, 204-001..010).</t>
+          <t>Total: 53 dokumen Martabe (51 baris; 0039/0040 dan 0041/0042 digabung per baris); 52 SWI diperiksa (201-001..025, 203-001..012, 204-001..015).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Martabe reference matrix with SWI 204-016..019
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0121qocWgsZdFAsne2oz9sHT
</commit_message>
<xml_diff>
--- a/Matriks-Rujukan-Martabe-SWI-201-203.xlsx
+++ b/Matriks-Rujukan-Martabe-SWI-201-203.xlsx
@@ -1719,7 +1719,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>204-002</t>
+          <t>204-002, 204-016</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2014,7 +2014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2222,6 +2222,42 @@
       <c r="B17" t="inlineStr">
         <is>
           <t>Hanya rujukan vendor (control philosophy Roytec); tidak ada rujukan SOP Martabe</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>204-017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Tidak ada prosedur pembersihan/verifikasi aperture sebelum revisi ini; hanya quotation ILS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>204-018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Hanya quotation ILS; tidak ada rujukan SOP Martabe</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>204-019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Tidak ada prosedur untuk instrumen ini sebelum revisi ini; hanya quotation ILS</t>
         </is>
       </c>
     </row>
@@ -2287,7 +2323,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Total: 53 dokumen Martabe (51 baris; 0039/0040 dan 0041/0042 digabung per baris); 52 SWI diperiksa (201-001..025, 203-001..012, 204-001..015).</t>
+          <t>Total: 53 dokumen Martabe (51 baris; 0039/0040 dan 0041/0042 digabung per baris); 56 SWI diperiksa (201-001..025, 203-001..012, 204-001..019).</t>
         </is>
       </c>
     </row>

</xml_diff>